<commit_message>
Add detailed revenue breakdown sheets to projection model
Added 3 new sheets (悲観的_詳細, 標準_詳細, 楽観的_詳細) with:
- Catalog requests: unit count × weighted avg unit price = revenue
- Event reservations: unit count × weighted avg unit price = revenue
- Housing contracts: count × avg price × commission rate × recovery rate = revenue
- Monthly listing fees
- Annual totals for all line items
- Plan mix details (成果報酬/掲載ベーシック/掲載プロ composition ratios)
- Weighted average unit prices calculated from plan mix

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/payhome_kagoshima_projection.xlsx
+++ b/docs/payhome_kagoshima_projection.xlsx
@@ -13,6 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="楽観的シナリオ" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3シナリオ比較" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="売上推移データ" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="悲観的_詳細" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="標準_詳細" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="楽観的_詳細" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,8 +24,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="9">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="¥#,##0"/>
+  </numFmts>
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,6 +78,18 @@
       <color rgb="002980B9"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E4057"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -111,7 +129,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -133,11 +151,55 @@
         <color rgb="00D5D8DC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5D8DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D8DC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5D8DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D8DC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -224,6 +286,51 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -302,7 +409,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -494,7 +600,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -4510,6 +4615,8 @@
           <t>年間売上1,362万円。月間売上200万円超（12月時点）。鹿児島県内26社掲載で平屋検討者の主要接点になれる水準。YouTube既知契約の約87%増の上乗せ効果。事業として成立する最低ラインをクリア。</t>
         </is>
       </c>
+      <c r="C27" s="36" t="n"/>
+      <c r="D27" s="37" t="n"/>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
@@ -4522,8 +4629,8 @@
           <t>月間固定費を50万円と仮定した場合、有料掲載社数10社＋月間リード15件で黒字化。標準シナリオでは9月（有料化2ヶ月目）に到達見込み。</t>
         </is>
       </c>
-      <c r="C28" s="17" t="n"/>
-      <c r="D28" s="17" t="n"/>
+      <c r="C28" s="36" t="n"/>
+      <c r="D28" s="37" t="n"/>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -4536,6 +4643,8 @@
           <t>鹿児島県内の平屋対応工務店は最大100〜150社。掲載率50%で50〜75社が上限。ARPUを上げるか、エリアを九州全域に拡大する必要あり。</t>
         </is>
       </c>
+      <c r="C29" s="36" t="n"/>
+      <c r="D29" s="37" t="n"/>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
@@ -4548,8 +4657,8 @@
           <t>既に年間10〜20棟の契約実績がある。PF化により送客精度が上がるため、標準シナリオ（+87%）は十分に現実的。</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
+      <c r="C30" s="36" t="n"/>
+      <c r="D30" s="37" t="n"/>
     </row>
     <row r="31" ht="60" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -4562,6 +4671,8 @@
           <t>フリープラン後の離脱率、成約報酬の回収率、工務店の対応品質が売上に直結。消費者フォローの仕組みが成約追跡の鍵。</t>
         </is>
       </c>
+      <c r="C31" s="36" t="n"/>
+      <c r="D31" s="37" t="n"/>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
@@ -4574,8 +4685,8 @@
           <t>鹿児島で実績を作った後、熊本・宮崎・福岡へ段階的に展開。九州全域で掲載100社＋マーケ支援20社で年商1億円が視野に入る。</t>
         </is>
       </c>
-      <c r="C32" s="17" t="n"/>
-      <c r="D32" s="17" t="n"/>
+      <c r="C32" s="36" t="n"/>
+      <c r="D32" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -4952,4 +5063,2995 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E74C3C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>悲観的シナリオ — 収益詳細（件数×単価）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>指標</t>
+        </is>
+      </c>
+      <c r="B3" s="39" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="D3" s="39" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="E3" s="39" t="inlineStr">
+        <is>
+          <t>7月</t>
+        </is>
+      </c>
+      <c r="F3" s="39" t="inlineStr">
+        <is>
+          <t>8月</t>
+        </is>
+      </c>
+      <c r="G3" s="39" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="H3" s="39" t="inlineStr">
+        <is>
+          <t>10月</t>
+        </is>
+      </c>
+      <c r="I3" s="39" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="J3" s="39" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="K3" s="39" t="inlineStr">
+        <is>
+          <t>1月</t>
+        </is>
+      </c>
+      <c r="L3" s="39" t="inlineStr">
+        <is>
+          <t>2月</t>
+        </is>
+      </c>
+      <c r="M3" s="39" t="inlineStr">
+        <is>
+          <t>3月</t>
+        </is>
+      </c>
+      <c r="N3" s="39" t="inlineStr">
+        <is>
+          <t>年間合計</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>有料掲載社数</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="J4" s="40" t="n">
+        <v>7</v>
+      </c>
+      <c r="K4" s="40" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" s="40" t="n">
+        <v>9</v>
+      </c>
+      <c r="M4" s="40" t="n">
+        <v>10</v>
+      </c>
+      <c r="N4" s="40" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>【資料請求】</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  件数</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" s="40" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 単価（加重平均 ¥6,600）</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>6600</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>6600</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>6600</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>6600</v>
+      </c>
+      <c r="J8" s="19" t="n">
+        <v>6600</v>
+      </c>
+      <c r="K8" s="19" t="n">
+        <v>6600</v>
+      </c>
+      <c r="L8" s="19" t="n">
+        <v>6600</v>
+      </c>
+      <c r="M8" s="19" t="n">
+        <v>6600</v>
+      </c>
+      <c r="N8" s="19" t="n">
+        <v>52800</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＝ 資料請求収益</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>6600</v>
+      </c>
+      <c r="G9" s="40" t="n">
+        <v>6600</v>
+      </c>
+      <c r="H9" s="40" t="n">
+        <v>13200</v>
+      </c>
+      <c r="I9" s="40" t="n">
+        <v>13200</v>
+      </c>
+      <c r="J9" s="40" t="n">
+        <v>13200</v>
+      </c>
+      <c r="K9" s="40" t="n">
+        <v>13200</v>
+      </c>
+      <c r="L9" s="40" t="n">
+        <v>19800</v>
+      </c>
+      <c r="M9" s="40" t="n">
+        <v>19800</v>
+      </c>
+      <c r="N9" s="40" t="n">
+        <v>105600</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>【見学会来場】</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  件数</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" s="40" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 単価（加重平均 ¥66,000）</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>66000</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>66000</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>66000</v>
+      </c>
+      <c r="J13" s="19" t="n">
+        <v>66000</v>
+      </c>
+      <c r="K13" s="19" t="n">
+        <v>66000</v>
+      </c>
+      <c r="L13" s="19" t="n">
+        <v>66000</v>
+      </c>
+      <c r="M13" s="19" t="n">
+        <v>66000</v>
+      </c>
+      <c r="N13" s="19" t="n">
+        <v>528000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＝ 見学会来場収益</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="40" t="n">
+        <v>66000</v>
+      </c>
+      <c r="G14" s="40" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H14" s="40" t="n">
+        <v>66000</v>
+      </c>
+      <c r="I14" s="40" t="n">
+        <v>66000</v>
+      </c>
+      <c r="J14" s="40" t="n">
+        <v>132000</v>
+      </c>
+      <c r="K14" s="40" t="n">
+        <v>132000</v>
+      </c>
+      <c r="L14" s="40" t="n">
+        <v>132000</v>
+      </c>
+      <c r="M14" s="40" t="n">
+        <v>132000</v>
+      </c>
+      <c r="N14" s="40" t="n">
+        <v>792000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>【住宅契約成約】</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  成約件数</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="40" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 平均契約金額 ¥2,200万円</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="H18" s="19" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="K18" s="19" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="L18" s="19" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="M18" s="19" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="N18" s="19" t="n">
+        <v>176000000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 報酬率（加重平均 3.5%）</t>
+        </is>
+      </c>
+      <c r="B19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="41" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="G19" s="41" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="H19" s="41" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="I19" s="41" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="J19" s="41" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="K19" s="41" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="L19" s="41" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="M19" s="41" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="N19" s="41" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 回収率（50%）</t>
+        </is>
+      </c>
+      <c r="B20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G20" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H20" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I20" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J20" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K20" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L20" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M20" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N20" s="42" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＝ 成約報酬収益</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="40" t="n">
+        <v>385000</v>
+      </c>
+      <c r="J21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="40" t="n">
+        <v>385000</v>
+      </c>
+      <c r="L21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="40" t="n">
+        <v>385000</v>
+      </c>
+      <c r="N21" s="40" t="n">
+        <v>1155000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>【月額掲載料】</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  月額掲載料</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="40" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G24" s="40" t="n">
+        <v>80000</v>
+      </c>
+      <c r="H24" s="40" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I24" s="40" t="n">
+        <v>120000</v>
+      </c>
+      <c r="J24" s="40" t="n">
+        <v>140000</v>
+      </c>
+      <c r="K24" s="40" t="n">
+        <v>160000</v>
+      </c>
+      <c r="L24" s="40" t="n">
+        <v>180000</v>
+      </c>
+      <c r="M24" s="40" t="n">
+        <v>200000</v>
+      </c>
+      <c r="N24" s="40" t="n">
+        <v>1040000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="43" t="inlineStr">
+        <is>
+          <t>月間売上合計</t>
+        </is>
+      </c>
+      <c r="B26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="44" t="n">
+        <v>132600</v>
+      </c>
+      <c r="G26" s="44" t="n">
+        <v>152600</v>
+      </c>
+      <c r="H26" s="44" t="n">
+        <v>179200</v>
+      </c>
+      <c r="I26" s="44" t="n">
+        <v>584200</v>
+      </c>
+      <c r="J26" s="44" t="n">
+        <v>285200</v>
+      </c>
+      <c r="K26" s="44" t="n">
+        <v>690200</v>
+      </c>
+      <c r="L26" s="44" t="n">
+        <v>331800</v>
+      </c>
+      <c r="M26" s="44" t="n">
+        <v>736800</v>
+      </c>
+      <c r="N26" s="44" t="n">
+        <v>3092600</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="43" t="inlineStr">
+        <is>
+          <t>累計売上</t>
+        </is>
+      </c>
+      <c r="B27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="44" t="n">
+        <v>132600</v>
+      </c>
+      <c r="G27" s="44" t="n">
+        <v>285200</v>
+      </c>
+      <c r="H27" s="44" t="n">
+        <v>464400</v>
+      </c>
+      <c r="I27" s="44" t="n">
+        <v>1048600</v>
+      </c>
+      <c r="J27" s="44" t="n">
+        <v>1333800</v>
+      </c>
+      <c r="K27" s="44" t="n">
+        <v>2024000</v>
+      </c>
+      <c r="L27" s="44" t="n">
+        <v>2355800</v>
+      </c>
+      <c r="M27" s="44" t="n">
+        <v>3092600</v>
+      </c>
+      <c r="N27" s="44" t="n">
+        <v>10737000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>【年間件数サマリー】</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  資料請求 合計件数</t>
+        </is>
+      </c>
+      <c r="N30" s="40" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  見学会来場 合計件数</t>
+        </is>
+      </c>
+      <c r="N31" s="40" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  成約 合計件数</t>
+        </is>
+      </c>
+      <c r="N32" s="40" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>単価設定の詳細（プラン構成比による加重平均）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="39" t="inlineStr">
+        <is>
+          <t>プラン</t>
+        </is>
+      </c>
+      <c r="B36" s="39" t="inlineStr">
+        <is>
+          <t>構成比</t>
+        </is>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>資料請求単価</t>
+        </is>
+      </c>
+      <c r="D36" s="39" t="inlineStr">
+        <is>
+          <t>見学会単価</t>
+        </is>
+      </c>
+      <c r="E36" s="39" t="inlineStr">
+        <is>
+          <t>成約報酬率</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="45" t="inlineStr">
+        <is>
+          <t>成果報酬</t>
+        </is>
+      </c>
+      <c r="B37" s="46" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C37" s="47" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D37" s="47" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E37" s="48" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="45" t="inlineStr">
+        <is>
+          <t>掲載ベーシック</t>
+        </is>
+      </c>
+      <c r="B38" s="46" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C38" s="47" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D38" s="47" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E38" s="48" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="45" t="inlineStr">
+        <is>
+          <t>掲載プロ</t>
+        </is>
+      </c>
+      <c r="B39" s="46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C39" s="47" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D39" s="47" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E39" s="48" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>加重平均</t>
+        </is>
+      </c>
+      <c r="B40" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="51" t="n">
+        <v>6600</v>
+      </c>
+      <c r="D40" s="51" t="n">
+        <v>66000</v>
+      </c>
+      <c r="E40" s="52" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0027AE60"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>標準シナリオ — 収益詳細（件数×単価）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>指標</t>
+        </is>
+      </c>
+      <c r="B3" s="39" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="D3" s="39" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="E3" s="39" t="inlineStr">
+        <is>
+          <t>7月</t>
+        </is>
+      </c>
+      <c r="F3" s="39" t="inlineStr">
+        <is>
+          <t>8月</t>
+        </is>
+      </c>
+      <c r="G3" s="39" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="H3" s="39" t="inlineStr">
+        <is>
+          <t>10月</t>
+        </is>
+      </c>
+      <c r="I3" s="39" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="J3" s="39" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="K3" s="39" t="inlineStr">
+        <is>
+          <t>1月</t>
+        </is>
+      </c>
+      <c r="L3" s="39" t="inlineStr">
+        <is>
+          <t>2月</t>
+        </is>
+      </c>
+      <c r="M3" s="39" t="inlineStr">
+        <is>
+          <t>3月</t>
+        </is>
+      </c>
+      <c r="N3" s="39" t="inlineStr">
+        <is>
+          <t>年間合計</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>有料掲載社数</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="40" t="n">
+        <v>12</v>
+      </c>
+      <c r="G4" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="H4" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="I4" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="J4" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="K4" s="40" t="n">
+        <v>22</v>
+      </c>
+      <c r="L4" s="40" t="n">
+        <v>24</v>
+      </c>
+      <c r="M4" s="40" t="n">
+        <v>26</v>
+      </c>
+      <c r="N4" s="40" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>【資料請求】</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  件数</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>11</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <v>13</v>
+      </c>
+      <c r="H7" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="I7" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="J7" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="K7" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="L7" s="40" t="n">
+        <v>22</v>
+      </c>
+      <c r="M7" s="40" t="n">
+        <v>23</v>
+      </c>
+      <c r="N7" s="40" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 単価（加重平均 ¥5,300）</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>5300</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>5300</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>5300</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>5300</v>
+      </c>
+      <c r="J8" s="19" t="n">
+        <v>5300</v>
+      </c>
+      <c r="K8" s="19" t="n">
+        <v>5300</v>
+      </c>
+      <c r="L8" s="19" t="n">
+        <v>5300</v>
+      </c>
+      <c r="M8" s="19" t="n">
+        <v>5300</v>
+      </c>
+      <c r="N8" s="19" t="n">
+        <v>42400</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＝ 資料請求収益</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>58300</v>
+      </c>
+      <c r="G9" s="40" t="n">
+        <v>68900</v>
+      </c>
+      <c r="H9" s="40" t="n">
+        <v>74200</v>
+      </c>
+      <c r="I9" s="40" t="n">
+        <v>84800</v>
+      </c>
+      <c r="J9" s="40" t="n">
+        <v>95400</v>
+      </c>
+      <c r="K9" s="40" t="n">
+        <v>106000</v>
+      </c>
+      <c r="L9" s="40" t="n">
+        <v>116600</v>
+      </c>
+      <c r="M9" s="40" t="n">
+        <v>121900</v>
+      </c>
+      <c r="N9" s="40" t="n">
+        <v>726100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>【見学会来場】</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  件数</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="40" t="n">
+        <v>7</v>
+      </c>
+      <c r="G12" s="40" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" s="40" t="n">
+        <v>10</v>
+      </c>
+      <c r="I12" s="40" t="n">
+        <v>11</v>
+      </c>
+      <c r="J12" s="40" t="n">
+        <v>12</v>
+      </c>
+      <c r="K12" s="40" t="n">
+        <v>13</v>
+      </c>
+      <c r="L12" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="M12" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="N12" s="40" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 単価（加重平均 ¥53,000）</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>53000</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>53000</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>53000</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>53000</v>
+      </c>
+      <c r="J13" s="19" t="n">
+        <v>53000</v>
+      </c>
+      <c r="K13" s="19" t="n">
+        <v>53000</v>
+      </c>
+      <c r="L13" s="19" t="n">
+        <v>53000</v>
+      </c>
+      <c r="M13" s="19" t="n">
+        <v>53000</v>
+      </c>
+      <c r="N13" s="19" t="n">
+        <v>424000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＝ 見学会来場収益</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="40" t="n">
+        <v>371000</v>
+      </c>
+      <c r="G14" s="40" t="n">
+        <v>424000</v>
+      </c>
+      <c r="H14" s="40" t="n">
+        <v>530000</v>
+      </c>
+      <c r="I14" s="40" t="n">
+        <v>583000</v>
+      </c>
+      <c r="J14" s="40" t="n">
+        <v>636000</v>
+      </c>
+      <c r="K14" s="40" t="n">
+        <v>689000</v>
+      </c>
+      <c r="L14" s="40" t="n">
+        <v>742000</v>
+      </c>
+      <c r="M14" s="40" t="n">
+        <v>848000</v>
+      </c>
+      <c r="N14" s="40" t="n">
+        <v>4823000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>【住宅契約成約】</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  成約件数</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="L17" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="M17" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="N17" s="40" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 平均契約金額 ¥2,500万円</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="H18" s="19" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="K18" s="19" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="L18" s="19" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="M18" s="19" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="N18" s="19" t="n">
+        <v>200000000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 報酬率（加重平均 3.0%）</t>
+        </is>
+      </c>
+      <c r="B19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="41" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G19" s="41" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H19" s="41" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I19" s="41" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J19" s="41" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K19" s="41" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L19" s="41" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M19" s="41" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N19" s="41" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 回収率（70%）</t>
+        </is>
+      </c>
+      <c r="B20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="42" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G20" s="42" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H20" s="42" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I20" s="42" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J20" s="42" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K20" s="42" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L20" s="42" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="M20" s="42" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="N20" s="42" t="n">
+        <v>5.600000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＝ 成約報酬収益</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="40" t="n">
+        <v>525000</v>
+      </c>
+      <c r="G21" s="40" t="n">
+        <v>525000</v>
+      </c>
+      <c r="H21" s="40" t="n">
+        <v>525000</v>
+      </c>
+      <c r="I21" s="40" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="J21" s="40" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="K21" s="40" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="L21" s="40" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="M21" s="40" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="N21" s="40" t="n">
+        <v>6825000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>【月額掲載料】</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  月額掲載料</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="40" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G24" s="40" t="n">
+        <v>240000</v>
+      </c>
+      <c r="H24" s="40" t="n">
+        <v>280000</v>
+      </c>
+      <c r="I24" s="40" t="n">
+        <v>320000</v>
+      </c>
+      <c r="J24" s="40" t="n">
+        <v>360000</v>
+      </c>
+      <c r="K24" s="40" t="n">
+        <v>400000</v>
+      </c>
+      <c r="L24" s="40" t="n">
+        <v>440000</v>
+      </c>
+      <c r="M24" s="40" t="n">
+        <v>480000</v>
+      </c>
+      <c r="N24" s="40" t="n">
+        <v>2720000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="43" t="inlineStr">
+        <is>
+          <t>月間売上合計</t>
+        </is>
+      </c>
+      <c r="B26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="44" t="n">
+        <v>1154300</v>
+      </c>
+      <c r="G26" s="44" t="n">
+        <v>1257900</v>
+      </c>
+      <c r="H26" s="44" t="n">
+        <v>1409200</v>
+      </c>
+      <c r="I26" s="44" t="n">
+        <v>2037800</v>
+      </c>
+      <c r="J26" s="44" t="n">
+        <v>2141400</v>
+      </c>
+      <c r="K26" s="44" t="n">
+        <v>2245000</v>
+      </c>
+      <c r="L26" s="44" t="n">
+        <v>2348600</v>
+      </c>
+      <c r="M26" s="44" t="n">
+        <v>2499900</v>
+      </c>
+      <c r="N26" s="44" t="n">
+        <v>15094100</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="43" t="inlineStr">
+        <is>
+          <t>累計売上</t>
+        </is>
+      </c>
+      <c r="B27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="44" t="n">
+        <v>1154300</v>
+      </c>
+      <c r="G27" s="44" t="n">
+        <v>2412200</v>
+      </c>
+      <c r="H27" s="44" t="n">
+        <v>3821400</v>
+      </c>
+      <c r="I27" s="44" t="n">
+        <v>5859200</v>
+      </c>
+      <c r="J27" s="44" t="n">
+        <v>8000600</v>
+      </c>
+      <c r="K27" s="44" t="n">
+        <v>10245600</v>
+      </c>
+      <c r="L27" s="44" t="n">
+        <v>12594200</v>
+      </c>
+      <c r="M27" s="44" t="n">
+        <v>15094100</v>
+      </c>
+      <c r="N27" s="44" t="n">
+        <v>59181600</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>【年間件数サマリー】</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  資料請求 合計件数</t>
+        </is>
+      </c>
+      <c r="N30" s="40" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  見学会来場 合計件数</t>
+        </is>
+      </c>
+      <c r="N31" s="40" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  成約 合計件数</t>
+        </is>
+      </c>
+      <c r="N32" s="40" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>単価設定の詳細（プラン構成比による加重平均）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="39" t="inlineStr">
+        <is>
+          <t>プラン</t>
+        </is>
+      </c>
+      <c r="B36" s="39" t="inlineStr">
+        <is>
+          <t>構成比</t>
+        </is>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>資料請求単価</t>
+        </is>
+      </c>
+      <c r="D36" s="39" t="inlineStr">
+        <is>
+          <t>見学会単価</t>
+        </is>
+      </c>
+      <c r="E36" s="39" t="inlineStr">
+        <is>
+          <t>成約報酬率</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="45" t="inlineStr">
+        <is>
+          <t>成果報酬</t>
+        </is>
+      </c>
+      <c r="B37" s="46" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C37" s="47" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D37" s="47" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E37" s="48" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="45" t="inlineStr">
+        <is>
+          <t>掲載ベーシック</t>
+        </is>
+      </c>
+      <c r="B38" s="46" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C38" s="47" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D38" s="47" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E38" s="48" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="45" t="inlineStr">
+        <is>
+          <t>掲載プロ</t>
+        </is>
+      </c>
+      <c r="B39" s="46" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C39" s="47" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D39" s="47" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E39" s="48" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>加重平均</t>
+        </is>
+      </c>
+      <c r="B40" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="51" t="n">
+        <v>5300</v>
+      </c>
+      <c r="D40" s="51" t="n">
+        <v>53000</v>
+      </c>
+      <c r="E40" s="52" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002980B9"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>楽観的シナリオ — 収益詳細（件数×単価）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>指標</t>
+        </is>
+      </c>
+      <c r="B3" s="39" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="D3" s="39" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="E3" s="39" t="inlineStr">
+        <is>
+          <t>7月</t>
+        </is>
+      </c>
+      <c r="F3" s="39" t="inlineStr">
+        <is>
+          <t>8月</t>
+        </is>
+      </c>
+      <c r="G3" s="39" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="H3" s="39" t="inlineStr">
+        <is>
+          <t>10月</t>
+        </is>
+      </c>
+      <c r="I3" s="39" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="J3" s="39" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="K3" s="39" t="inlineStr">
+        <is>
+          <t>1月</t>
+        </is>
+      </c>
+      <c r="L3" s="39" t="inlineStr">
+        <is>
+          <t>2月</t>
+        </is>
+      </c>
+      <c r="M3" s="39" t="inlineStr">
+        <is>
+          <t>3月</t>
+        </is>
+      </c>
+      <c r="N3" s="39" t="inlineStr">
+        <is>
+          <t>年間合計</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>有料掲載社数</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="40" t="n">
+        <v>22</v>
+      </c>
+      <c r="G4" s="40" t="n">
+        <v>25</v>
+      </c>
+      <c r="H4" s="40" t="n">
+        <v>28</v>
+      </c>
+      <c r="I4" s="40" t="n">
+        <v>31</v>
+      </c>
+      <c r="J4" s="40" t="n">
+        <v>34</v>
+      </c>
+      <c r="K4" s="40" t="n">
+        <v>37</v>
+      </c>
+      <c r="L4" s="40" t="n">
+        <v>40</v>
+      </c>
+      <c r="M4" s="40" t="n">
+        <v>43</v>
+      </c>
+      <c r="N4" s="40" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>【資料請求】</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  件数</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>40</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <v>45</v>
+      </c>
+      <c r="H7" s="40" t="n">
+        <v>50</v>
+      </c>
+      <c r="I7" s="40" t="n">
+        <v>56</v>
+      </c>
+      <c r="J7" s="40" t="n">
+        <v>61</v>
+      </c>
+      <c r="K7" s="40" t="n">
+        <v>67</v>
+      </c>
+      <c r="L7" s="40" t="n">
+        <v>72</v>
+      </c>
+      <c r="M7" s="40" t="n">
+        <v>77</v>
+      </c>
+      <c r="N7" s="40" t="n">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 単価（加重平均 ¥4,600）</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>4600</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>4600</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>4600</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>4600</v>
+      </c>
+      <c r="J8" s="19" t="n">
+        <v>4600</v>
+      </c>
+      <c r="K8" s="19" t="n">
+        <v>4600</v>
+      </c>
+      <c r="L8" s="19" t="n">
+        <v>4600</v>
+      </c>
+      <c r="M8" s="19" t="n">
+        <v>4600</v>
+      </c>
+      <c r="N8" s="19" t="n">
+        <v>36800</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＝ 資料請求収益</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>184000</v>
+      </c>
+      <c r="G9" s="40" t="n">
+        <v>207000</v>
+      </c>
+      <c r="H9" s="40" t="n">
+        <v>230000</v>
+      </c>
+      <c r="I9" s="40" t="n">
+        <v>257600</v>
+      </c>
+      <c r="J9" s="40" t="n">
+        <v>280600</v>
+      </c>
+      <c r="K9" s="40" t="n">
+        <v>308200</v>
+      </c>
+      <c r="L9" s="40" t="n">
+        <v>331200</v>
+      </c>
+      <c r="M9" s="40" t="n">
+        <v>354200</v>
+      </c>
+      <c r="N9" s="40" t="n">
+        <v>2152800</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>【見学会来場】</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  件数</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="40" t="n">
+        <v>26</v>
+      </c>
+      <c r="G12" s="40" t="n">
+        <v>30</v>
+      </c>
+      <c r="H12" s="40" t="n">
+        <v>34</v>
+      </c>
+      <c r="I12" s="40" t="n">
+        <v>37</v>
+      </c>
+      <c r="J12" s="40" t="n">
+        <v>41</v>
+      </c>
+      <c r="K12" s="40" t="n">
+        <v>44</v>
+      </c>
+      <c r="L12" s="40" t="n">
+        <v>48</v>
+      </c>
+      <c r="M12" s="40" t="n">
+        <v>52</v>
+      </c>
+      <c r="N12" s="40" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 単価（加重平均 ¥46,000）</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>46000</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>46000</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>46000</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>46000</v>
+      </c>
+      <c r="J13" s="19" t="n">
+        <v>46000</v>
+      </c>
+      <c r="K13" s="19" t="n">
+        <v>46000</v>
+      </c>
+      <c r="L13" s="19" t="n">
+        <v>46000</v>
+      </c>
+      <c r="M13" s="19" t="n">
+        <v>46000</v>
+      </c>
+      <c r="N13" s="19" t="n">
+        <v>368000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＝ 見学会来場収益</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="40" t="n">
+        <v>1196000</v>
+      </c>
+      <c r="G14" s="40" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="H14" s="40" t="n">
+        <v>1564000</v>
+      </c>
+      <c r="I14" s="40" t="n">
+        <v>1702000</v>
+      </c>
+      <c r="J14" s="40" t="n">
+        <v>1886000</v>
+      </c>
+      <c r="K14" s="40" t="n">
+        <v>2024000</v>
+      </c>
+      <c r="L14" s="40" t="n">
+        <v>2208000</v>
+      </c>
+      <c r="M14" s="40" t="n">
+        <v>2392000</v>
+      </c>
+      <c r="N14" s="40" t="n">
+        <v>14352000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>【住宅契約成約】</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  成約件数</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="40" t="n">
+        <v>7</v>
+      </c>
+      <c r="I17" s="40" t="n">
+        <v>7</v>
+      </c>
+      <c r="J17" s="40" t="n">
+        <v>8</v>
+      </c>
+      <c r="K17" s="40" t="n">
+        <v>9</v>
+      </c>
+      <c r="L17" s="40" t="n">
+        <v>10</v>
+      </c>
+      <c r="M17" s="40" t="n">
+        <v>10</v>
+      </c>
+      <c r="N17" s="40" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 平均契約金額 ¥2,800万円</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="H18" s="19" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="K18" s="19" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="L18" s="19" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="M18" s="19" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="N18" s="19" t="n">
+        <v>224000000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 報酬率（加重平均 2.7%）</t>
+        </is>
+      </c>
+      <c r="B19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="41" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="G19" s="41" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="H19" s="41" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="I19" s="41" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="J19" s="41" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="K19" s="41" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="L19" s="41" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="M19" s="41" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="N19" s="41" t="n">
+        <v>0.216</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × 回収率（90%）</t>
+        </is>
+      </c>
+      <c r="B20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="42" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G20" s="42" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H20" s="42" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I20" s="42" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J20" s="42" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K20" s="42" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L20" s="42" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M20" s="42" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="N20" s="42" t="n">
+        <v>7.200000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＝ 成約報酬収益</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="40" t="n">
+        <v>3402000</v>
+      </c>
+      <c r="G21" s="40" t="n">
+        <v>4082400</v>
+      </c>
+      <c r="H21" s="40" t="n">
+        <v>4762800</v>
+      </c>
+      <c r="I21" s="40" t="n">
+        <v>4762800</v>
+      </c>
+      <c r="J21" s="40" t="n">
+        <v>5443200</v>
+      </c>
+      <c r="K21" s="40" t="n">
+        <v>6123600</v>
+      </c>
+      <c r="L21" s="40" t="n">
+        <v>6804000</v>
+      </c>
+      <c r="M21" s="40" t="n">
+        <v>6804000</v>
+      </c>
+      <c r="N21" s="40" t="n">
+        <v>42184800</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>【月額掲載料】</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  月額掲載料</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="40" t="n">
+        <v>440000</v>
+      </c>
+      <c r="G24" s="40" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H24" s="40" t="n">
+        <v>560000</v>
+      </c>
+      <c r="I24" s="40" t="n">
+        <v>620000</v>
+      </c>
+      <c r="J24" s="40" t="n">
+        <v>680000</v>
+      </c>
+      <c r="K24" s="40" t="n">
+        <v>740000</v>
+      </c>
+      <c r="L24" s="40" t="n">
+        <v>800000</v>
+      </c>
+      <c r="M24" s="40" t="n">
+        <v>860000</v>
+      </c>
+      <c r="N24" s="40" t="n">
+        <v>5200000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="43" t="inlineStr">
+        <is>
+          <t>月間売上合計</t>
+        </is>
+      </c>
+      <c r="B26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="44" t="n">
+        <v>5222000</v>
+      </c>
+      <c r="G26" s="44" t="n">
+        <v>6169400</v>
+      </c>
+      <c r="H26" s="44" t="n">
+        <v>7116800</v>
+      </c>
+      <c r="I26" s="44" t="n">
+        <v>7342400</v>
+      </c>
+      <c r="J26" s="44" t="n">
+        <v>8289800</v>
+      </c>
+      <c r="K26" s="44" t="n">
+        <v>9195800</v>
+      </c>
+      <c r="L26" s="44" t="n">
+        <v>10143200</v>
+      </c>
+      <c r="M26" s="44" t="n">
+        <v>10410200</v>
+      </c>
+      <c r="N26" s="44" t="n">
+        <v>63889600</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="43" t="inlineStr">
+        <is>
+          <t>累計売上</t>
+        </is>
+      </c>
+      <c r="B27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="44" t="n">
+        <v>5222000</v>
+      </c>
+      <c r="G27" s="44" t="n">
+        <v>11391400</v>
+      </c>
+      <c r="H27" s="44" t="n">
+        <v>18508200</v>
+      </c>
+      <c r="I27" s="44" t="n">
+        <v>25850600</v>
+      </c>
+      <c r="J27" s="44" t="n">
+        <v>34140400</v>
+      </c>
+      <c r="K27" s="44" t="n">
+        <v>43336200</v>
+      </c>
+      <c r="L27" s="44" t="n">
+        <v>53479400</v>
+      </c>
+      <c r="M27" s="44" t="n">
+        <v>63889600</v>
+      </c>
+      <c r="N27" s="44" t="n">
+        <v>255817800</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>【年間件数サマリー】</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  資料請求 合計件数</t>
+        </is>
+      </c>
+      <c r="N30" s="40" t="n">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  見学会来場 合計件数</t>
+        </is>
+      </c>
+      <c r="N31" s="40" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  成約 合計件数</t>
+        </is>
+      </c>
+      <c r="N32" s="40" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>単価設定の詳細（プラン構成比による加重平均）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="39" t="inlineStr">
+        <is>
+          <t>プラン</t>
+        </is>
+      </c>
+      <c r="B36" s="39" t="inlineStr">
+        <is>
+          <t>構成比</t>
+        </is>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>資料請求単価</t>
+        </is>
+      </c>
+      <c r="D36" s="39" t="inlineStr">
+        <is>
+          <t>見学会単価</t>
+        </is>
+      </c>
+      <c r="E36" s="39" t="inlineStr">
+        <is>
+          <t>成約報酬率</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="45" t="inlineStr">
+        <is>
+          <t>成果報酬</t>
+        </is>
+      </c>
+      <c r="B37" s="46" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C37" s="47" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D37" s="47" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E37" s="48" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="45" t="inlineStr">
+        <is>
+          <t>掲載ベーシック</t>
+        </is>
+      </c>
+      <c r="B38" s="46" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C38" s="47" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D38" s="47" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E38" s="48" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="45" t="inlineStr">
+        <is>
+          <t>掲載プロ</t>
+        </is>
+      </c>
+      <c r="B39" s="46" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C39" s="47" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D39" s="47" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E39" s="48" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>加重平均</t>
+        </is>
+      </c>
+      <c r="B40" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="51" t="n">
+        <v>4600</v>
+      </c>
+      <c r="D40" s="51" t="n">
+        <v>46000</v>
+      </c>
+      <c r="E40" s="52" t="n">
+        <v>0.027</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>